<commit_message>
CrossFit: kombinace částí (AMRAP+EMOM), pomůcky podle formátu s anglickými názvy, 44 nových cviků
- hlavní část CrossFitu z více částí, každá s vlastním typem a časem
- pomůcky: formáty zobrazení, anglické názvy (BOX, dumbbell, barbell...), nové: rings, sled, bench, GHD, rope
- BOSU, lano, roller, stepper a TRX se v CrossFitu nenabízejí
- admin: úprava pomůcek
- knihovna: 191 cviků, migrace 0002

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/cviky_import.xlsx
+++ b/docs/cviky_import.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Kontrola" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cviky'!$A$1:$N$148</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cviky'!$A$1:$N$192</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -453,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N148"/>
+  <dimension ref="A1:N192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9952,8 +9952,2824 @@
         </is>
       </c>
     </row>
+    <row r="149">
+      <c r="A149" s="3" t="inlineStr">
+        <is>
+          <t>Přední dřep s osou</t>
+        </is>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>Front squat</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>nohy</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E149" s="3" t="inlineStr">
+        <is>
+          <t>osa</t>
+        </is>
+      </c>
+      <c r="F149" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G149" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H149" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I149" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J149" s="3" t="inlineStr">
+        <is>
+          <t>dřep</t>
+        </is>
+      </c>
+      <c r="K149" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L149" s="4" t="inlineStr">
+        <is>
+          <t>Osa leží na ramenou před krkem, lokty vpředu. Sedni do dřepu s rovným trupem.</t>
+        </is>
+      </c>
+      <c r="M149" s="3" t="n"/>
+      <c r="N149" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="3" t="inlineStr">
+        <is>
+          <t>Dřep s osou nad hlavou</t>
+        </is>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>Overhead squat</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>celé tělo</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="inlineStr">
+        <is>
+          <t>expert</t>
+        </is>
+      </c>
+      <c r="E150" s="3" t="inlineStr">
+        <is>
+          <t>osa</t>
+        </is>
+      </c>
+      <c r="F150" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G150" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H150" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I150" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J150" s="3" t="inlineStr">
+        <is>
+          <t>dřep</t>
+        </is>
+      </c>
+      <c r="K150" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="L150" s="4" t="inlineStr">
+        <is>
+          <t>Osu drž nad hlavou na širokém úchopu a sedni do hlubokého dřepu. Paže propnuté.</t>
+        </is>
+      </c>
+      <c r="M150" s="3" t="n"/>
+      <c r="N150" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="3" t="inlineStr">
+        <is>
+          <t>Push press</t>
+        </is>
+      </c>
+      <c r="B151" s="3" t="inlineStr">
+        <is>
+          <t>Push press</t>
+        </is>
+      </c>
+      <c r="C151" s="3" t="inlineStr">
+        <is>
+          <t>ramena</t>
+        </is>
+      </c>
+      <c r="D151" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E151" s="3" t="inlineStr">
+        <is>
+          <t>osa</t>
+        </is>
+      </c>
+      <c r="F151" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G151" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H151" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I151" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J151" s="3" t="inlineStr">
+        <is>
+          <t>tlak</t>
+        </is>
+      </c>
+      <c r="K151" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L151" s="4" t="inlineStr">
+        <is>
+          <t>Osa na ramenou, lehce poklekni a výbušně ji vytlač nad hlavu. Nahoře propni.</t>
+        </is>
+      </c>
+      <c r="M151" s="3" t="n"/>
+      <c r="N151" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="3" t="inlineStr">
+        <is>
+          <t>Zdvih osy na hrudník</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>Power clean</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>celé tělo</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E152" s="3" t="inlineStr">
+        <is>
+          <t>osa</t>
+        </is>
+      </c>
+      <c r="F152" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G152" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H152" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I152" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J152" s="3" t="inlineStr">
+        <is>
+          <t>jiné</t>
+        </is>
+      </c>
+      <c r="K152" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="L152" s="4" t="inlineStr">
+        <is>
+          <t>Osa u holení, výbušně natáhni kyčle a zachyť osu na ramenou. Lokty rychle dopředu.</t>
+        </is>
+      </c>
+      <c r="M152" s="3" t="n"/>
+      <c r="N152" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="3" t="inlineStr">
+        <is>
+          <t>Zdvih osy z visu na hrudník</t>
+        </is>
+      </c>
+      <c r="B153" s="3" t="inlineStr">
+        <is>
+          <t>Hang power clean</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>celé tělo</t>
+        </is>
+      </c>
+      <c r="D153" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E153" s="3" t="inlineStr">
+        <is>
+          <t>osa</t>
+        </is>
+      </c>
+      <c r="F153" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G153" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H153" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I153" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J153" s="3" t="inlineStr">
+        <is>
+          <t>jiné</t>
+        </is>
+      </c>
+      <c r="K153" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L153" s="4" t="inlineStr">
+        <is>
+          <t>Osa ve výši kolen, předkloň se a výbušně natáhni kyčle. Zachyť osu na ramenou.</t>
+        </is>
+      </c>
+      <c r="M153" s="3" t="n"/>
+      <c r="N153" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="3" t="inlineStr">
+        <is>
+          <t>Trh s osou</t>
+        </is>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>Barbell snatch</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>celé tělo</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="inlineStr">
+        <is>
+          <t>expert</t>
+        </is>
+      </c>
+      <c r="E154" s="3" t="inlineStr">
+        <is>
+          <t>osa</t>
+        </is>
+      </c>
+      <c r="F154" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G154" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H154" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I154" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J154" s="3" t="inlineStr">
+        <is>
+          <t>jiné</t>
+        </is>
+      </c>
+      <c r="K154" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="L154" s="4" t="inlineStr">
+        <is>
+          <t>Široký úchop, jedním plynulým pohybem vytáhni osu ze země nad hlavu. Zachyť ji v dřepu.</t>
+        </is>
+      </c>
+      <c r="M154" s="3" t="n"/>
+      <c r="N154" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="3" t="inlineStr">
+        <is>
+          <t>Nadhoz a vyražení osy</t>
+        </is>
+      </c>
+      <c r="B155" s="3" t="inlineStr">
+        <is>
+          <t>Clean and jerk</t>
+        </is>
+      </c>
+      <c r="C155" s="3" t="inlineStr">
+        <is>
+          <t>celé tělo</t>
+        </is>
+      </c>
+      <c r="D155" s="3" t="inlineStr">
+        <is>
+          <t>expert</t>
+        </is>
+      </c>
+      <c r="E155" s="3" t="inlineStr">
+        <is>
+          <t>osa</t>
+        </is>
+      </c>
+      <c r="F155" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G155" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H155" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I155" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J155" s="3" t="inlineStr">
+        <is>
+          <t>jiné</t>
+        </is>
+      </c>
+      <c r="K155" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="L155" s="4" t="inlineStr">
+        <is>
+          <t>Přenes osu na ramena a výbušně ji vyraž nad hlavu. Hýždě napnuté.</t>
+        </is>
+      </c>
+      <c r="M155" s="3" t="n"/>
+      <c r="N155" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="3" t="inlineStr">
+        <is>
+          <t>Thruster s osou</t>
+        </is>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>Barbell thruster</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>celé tělo</t>
+        </is>
+      </c>
+      <c r="D156" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E156" s="3" t="inlineStr">
+        <is>
+          <t>osa</t>
+        </is>
+      </c>
+      <c r="F156" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G156" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H156" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I156" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J156" s="3" t="inlineStr">
+        <is>
+          <t>dřep</t>
+        </is>
+      </c>
+      <c r="K156" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="L156" s="4" t="inlineStr">
+        <is>
+          <t>Osa na ramenou, sedni do dřepu a při vstávání ji vytlač nad hlavu. Plynule.</t>
+        </is>
+      </c>
+      <c r="M156" s="3" t="n"/>
+      <c r="N156" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="3" t="inlineStr">
+        <is>
+          <t>Veslování s osou</t>
+        </is>
+      </c>
+      <c r="B157" s="3" t="inlineStr">
+        <is>
+          <t>Barbell row</t>
+        </is>
+      </c>
+      <c r="C157" s="3" t="inlineStr">
+        <is>
+          <t>záda</t>
+        </is>
+      </c>
+      <c r="D157" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E157" s="3" t="inlineStr">
+        <is>
+          <t>osa</t>
+        </is>
+      </c>
+      <c r="F157" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G157" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H157" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I157" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J157" s="3" t="inlineStr">
+        <is>
+          <t>tah</t>
+        </is>
+      </c>
+      <c r="K157" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="L157" s="4" t="inlineStr">
+        <is>
+          <t>V předklonu přitáhni osu k pasu. Záda rovná, lopatky stáhni.</t>
+        </is>
+      </c>
+      <c r="M157" s="3" t="n"/>
+      <c r="N157" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t>Přitažení osy k bradě</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>Sumo deadlift high pull</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>celé tělo</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E158" s="3" t="inlineStr">
+        <is>
+          <t>osa</t>
+        </is>
+      </c>
+      <c r="F158" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G158" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H158" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I158" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J158" s="3" t="inlineStr">
+        <is>
+          <t>tah</t>
+        </is>
+      </c>
+      <c r="K158" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="L158" s="4" t="inlineStr">
+        <is>
+          <t>Široký rozkrok, zvedni osu a vytáhni ji lokty vysoko k bradě. Pohyb začíná v kyčlích.</t>
+        </is>
+      </c>
+      <c r="M158" s="3" t="n"/>
+      <c r="N158" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="3" t="inlineStr">
+        <is>
+          <t>Push jerk</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="inlineStr">
+        <is>
+          <t>Push jerk</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>ramena</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E159" s="3" t="inlineStr">
+        <is>
+          <t>osa</t>
+        </is>
+      </c>
+      <c r="F159" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G159" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H159" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I159" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J159" s="3" t="inlineStr">
+        <is>
+          <t>tlak</t>
+        </is>
+      </c>
+      <c r="K159" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="L159" s="4" t="inlineStr">
+        <is>
+          <t>Osa na ramenou, rychle poklekni a výbušně vyraž osu nad hlavu. Dopadni v mírném podřepu.</t>
+        </is>
+      </c>
+      <c r="M159" s="3" t="n"/>
+      <c r="N159" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="3" t="inlineStr">
+        <is>
+          <t>Tlak s osou vleže</t>
+        </is>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>Bench press</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>hrudník</t>
+        </is>
+      </c>
+      <c r="D160" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E160" s="3" t="inlineStr">
+        <is>
+          <t>osa, lavice</t>
+        </is>
+      </c>
+      <c r="F160" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G160" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H160" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I160" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J160" s="3" t="inlineStr">
+        <is>
+          <t>tlak</t>
+        </is>
+      </c>
+      <c r="K160" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L160" s="4" t="inlineStr">
+        <is>
+          <t>Vleže na lavici spusť osu k hrudi a vytlač zpět. Lopatky stáhni, chodidla pevně na zemi.</t>
+        </is>
+      </c>
+      <c r="M160" s="3" t="n"/>
+      <c r="N160" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="3" t="inlineStr">
+        <is>
+          <t>Tlak činek na lavici</t>
+        </is>
+      </c>
+      <c r="B161" s="3" t="inlineStr">
+        <is>
+          <t>Dumbbell bench press</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>hrudník</t>
+        </is>
+      </c>
+      <c r="D161" s="3" t="inlineStr">
+        <is>
+          <t>začátečník</t>
+        </is>
+      </c>
+      <c r="E161" s="3" t="inlineStr">
+        <is>
+          <t>činky, lavice</t>
+        </is>
+      </c>
+      <c r="F161" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G161" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H161" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I161" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J161" s="3" t="inlineStr">
+        <is>
+          <t>tlak</t>
+        </is>
+      </c>
+      <c r="K161" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="L161" s="4" t="inlineStr">
+        <is>
+          <t>Vleže na lavici vytlač činky nad hrudník. Spouštěj je pomalu.</t>
+        </is>
+      </c>
+      <c r="M161" s="3" t="n"/>
+      <c r="N161" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="3" t="inlineStr">
+        <is>
+          <t>Devil press</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>Devil press</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>celé tělo</t>
+        </is>
+      </c>
+      <c r="D162" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E162" s="3" t="inlineStr">
+        <is>
+          <t>činky</t>
+        </is>
+      </c>
+      <c r="F162" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G162" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H162" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I162" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J162" s="3" t="inlineStr">
+        <is>
+          <t>jiné</t>
+        </is>
+      </c>
+      <c r="K162" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L162" s="4" t="inlineStr">
+        <is>
+          <t>Klik na činkách, pak je jedním švihem přemísti nad hlavu. Zpět do kliku.</t>
+        </is>
+      </c>
+      <c r="M162" s="3" t="n"/>
+      <c r="N162" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="3" t="inlineStr">
+        <is>
+          <t>Zdvih činek na ramena a vytlačení</t>
+        </is>
+      </c>
+      <c r="B163" s="3" t="inlineStr">
+        <is>
+          <t>DB hang clean and jerk</t>
+        </is>
+      </c>
+      <c r="C163" s="3" t="inlineStr">
+        <is>
+          <t>celé tělo</t>
+        </is>
+      </c>
+      <c r="D163" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E163" s="3" t="inlineStr">
+        <is>
+          <t>činky</t>
+        </is>
+      </c>
+      <c r="F163" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G163" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H163" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I163" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J163" s="3" t="inlineStr">
+        <is>
+          <t>jiné</t>
+        </is>
+      </c>
+      <c r="K163" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="L163" s="4" t="inlineStr">
+        <is>
+          <t>Činky u stehen, výbušně je zachyť na ramenou a vytlač nad hlavu. Střídej ruce.</t>
+        </is>
+      </c>
+      <c r="M163" s="3" t="n"/>
+      <c r="N163" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="3" t="inlineStr">
+        <is>
+          <t>Výpady s činkami v chůzi</t>
+        </is>
+      </c>
+      <c r="B164" s="3" t="inlineStr">
+        <is>
+          <t>Dumbbell walking lunge</t>
+        </is>
+      </c>
+      <c r="C164" s="3" t="inlineStr">
+        <is>
+          <t>nohy</t>
+        </is>
+      </c>
+      <c r="D164" s="3" t="inlineStr">
+        <is>
+          <t>začátečník</t>
+        </is>
+      </c>
+      <c r="E164" s="3" t="inlineStr">
+        <is>
+          <t>činky</t>
+        </is>
+      </c>
+      <c r="F164" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G164" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H164" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I164" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J164" s="3" t="inlineStr">
+        <is>
+          <t>výpad</t>
+        </is>
+      </c>
+      <c r="K164" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="L164" s="4" t="inlineStr">
+        <is>
+          <t>S činkami v rukou jdi vpřed ve výpadech. Koleno nad kotníkem.</t>
+        </is>
+      </c>
+      <c r="M164" s="3" t="n"/>
+      <c r="N164" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="3" t="inlineStr">
+        <is>
+          <t>Rumunský mrtvý tah s činkami</t>
+        </is>
+      </c>
+      <c r="B165" s="3" t="inlineStr">
+        <is>
+          <t>Dumbbell Romanian deadlift</t>
+        </is>
+      </c>
+      <c r="C165" s="3" t="inlineStr">
+        <is>
+          <t>nohy</t>
+        </is>
+      </c>
+      <c r="D165" s="3" t="inlineStr">
+        <is>
+          <t>začátečník</t>
+        </is>
+      </c>
+      <c r="E165" s="3" t="inlineStr">
+        <is>
+          <t>činky</t>
+        </is>
+      </c>
+      <c r="F165" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G165" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H165" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I165" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J165" s="3" t="inlineStr">
+        <is>
+          <t>záklon/předklon</t>
+        </is>
+      </c>
+      <c r="K165" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="L165" s="4" t="inlineStr">
+        <is>
+          <t>Činky u stehen, sklop trup z kyčlí a vrať se. Záda rovná, kolena mírně pokrčená.</t>
+        </is>
+      </c>
+      <c r="M165" s="3" t="n"/>
+      <c r="N165" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="3" t="inlineStr">
+        <is>
+          <t>Přešlapy přes bednu s činkami</t>
+        </is>
+      </c>
+      <c r="B166" s="3" t="inlineStr">
+        <is>
+          <t>Dumbbell box step-over</t>
+        </is>
+      </c>
+      <c r="C166" s="3" t="inlineStr">
+        <is>
+          <t>nohy</t>
+        </is>
+      </c>
+      <c r="D166" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E166" s="3" t="inlineStr">
+        <is>
+          <t>bedna, činky</t>
+        </is>
+      </c>
+      <c r="F166" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G166" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H166" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I166" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J166" s="3" t="inlineStr">
+        <is>
+          <t>výpad</t>
+        </is>
+      </c>
+      <c r="K166" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="L166" s="4" t="inlineStr">
+        <is>
+          <t>Činky v rukou, našlápni na bednu a sestup na druhou stranu. Střídej nohy.</t>
+        </is>
+      </c>
+      <c r="M166" s="3" t="n"/>
+      <c r="N166" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="3" t="inlineStr">
+        <is>
+          <t>Veslování s činkami ve vzporu</t>
+        </is>
+      </c>
+      <c r="B167" s="3" t="inlineStr">
+        <is>
+          <t>Renegade row</t>
+        </is>
+      </c>
+      <c r="C167" s="3" t="inlineStr">
+        <is>
+          <t>záda</t>
+        </is>
+      </c>
+      <c r="D167" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E167" s="3" t="inlineStr">
+        <is>
+          <t>činky</t>
+        </is>
+      </c>
+      <c r="F167" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G167" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H167" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I167" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J167" s="3" t="inlineStr">
+        <is>
+          <t>tah</t>
+        </is>
+      </c>
+      <c r="K167" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L167" s="4" t="inlineStr">
+        <is>
+          <t>Ve vzporu na činkách přitahuj střídavě jednu činku k boku. Boky drž stabilní.</t>
+        </is>
+      </c>
+      <c r="M167" s="3" t="n"/>
+      <c r="N167" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="3" t="inlineStr">
+        <is>
+          <t>Zdvih kettlebellu a vytlačení</t>
+        </is>
+      </c>
+      <c r="B168" s="3" t="inlineStr">
+        <is>
+          <t>Kettlebell clean and press</t>
+        </is>
+      </c>
+      <c r="C168" s="3" t="inlineStr">
+        <is>
+          <t>ramena</t>
+        </is>
+      </c>
+      <c r="D168" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E168" s="3" t="inlineStr">
+        <is>
+          <t>kettlebell</t>
+        </is>
+      </c>
+      <c r="F168" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G168" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H168" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I168" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J168" s="3" t="inlineStr">
+        <is>
+          <t>tlak</t>
+        </is>
+      </c>
+      <c r="K168" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L168" s="4" t="inlineStr">
+        <is>
+          <t>Kettlebell vyzdvihni na rameno a vytlač nad hlavu. Střídej ruce.</t>
+        </is>
+      </c>
+      <c r="M168" s="3" t="n"/>
+      <c r="N168" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="3" t="inlineStr">
+        <is>
+          <t>Trh s kettlebellem</t>
+        </is>
+      </c>
+      <c r="B169" s="3" t="inlineStr">
+        <is>
+          <t>Kettlebell snatch</t>
+        </is>
+      </c>
+      <c r="C169" s="3" t="inlineStr">
+        <is>
+          <t>celé tělo</t>
+        </is>
+      </c>
+      <c r="D169" s="3" t="inlineStr">
+        <is>
+          <t>expert</t>
+        </is>
+      </c>
+      <c r="E169" s="3" t="inlineStr">
+        <is>
+          <t>kettlebell</t>
+        </is>
+      </c>
+      <c r="F169" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G169" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H169" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I169" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J169" s="3" t="inlineStr">
+        <is>
+          <t>jiné</t>
+        </is>
+      </c>
+      <c r="K169" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="L169" s="4" t="inlineStr">
+        <is>
+          <t>Švihni kettlebellem z kyčlí jedním pohybem nad hlavu. Zachyť ho na propnuté paži.</t>
+        </is>
+      </c>
+      <c r="M169" s="3" t="n"/>
+      <c r="N169" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="3" t="inlineStr">
+        <is>
+          <t>Americký švih s kettlebellem</t>
+        </is>
+      </c>
+      <c r="B170" s="3" t="inlineStr">
+        <is>
+          <t>American kettlebell swing</t>
+        </is>
+      </c>
+      <c r="C170" s="3" t="inlineStr">
+        <is>
+          <t>celé tělo</t>
+        </is>
+      </c>
+      <c r="D170" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E170" s="3" t="inlineStr">
+        <is>
+          <t>kettlebell</t>
+        </is>
+      </c>
+      <c r="F170" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G170" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H170" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I170" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J170" s="3" t="inlineStr">
+        <is>
+          <t>záklon/předklon</t>
+        </is>
+      </c>
+      <c r="K170" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="L170" s="4" t="inlineStr">
+        <is>
+          <t>Švihni kettlebellem až nad hlavu. Kyčle pohánějí pohyb, záda rovná.</t>
+        </is>
+      </c>
+      <c r="M170" s="3" t="n"/>
+      <c r="N170" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="3" t="inlineStr">
+        <is>
+          <t>Angličák s výskokem na bednu</t>
+        </is>
+      </c>
+      <c r="B171" s="3" t="inlineStr">
+        <is>
+          <t>Burpee box jump</t>
+        </is>
+      </c>
+      <c r="C171" s="3" t="inlineStr">
+        <is>
+          <t>celé tělo</t>
+        </is>
+      </c>
+      <c r="D171" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E171" s="3" t="inlineStr">
+        <is>
+          <t>bedna</t>
+        </is>
+      </c>
+      <c r="F171" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G171" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H171" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I171" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J171" s="3" t="inlineStr">
+        <is>
+          <t>skok</t>
+        </is>
+      </c>
+      <c r="K171" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L171" s="4" t="inlineStr">
+        <is>
+          <t>Angličák před bednou, po kliku vyskoč na bednu a vzpřimuj se. Sestup.</t>
+        </is>
+      </c>
+      <c r="M171" s="3" t="n"/>
+      <c r="N171" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="3" t="inlineStr">
+        <is>
+          <t>Přeskok bedny</t>
+        </is>
+      </c>
+      <c r="B172" s="3" t="inlineStr">
+        <is>
+          <t>Box jump over</t>
+        </is>
+      </c>
+      <c r="C172" s="3" t="inlineStr">
+        <is>
+          <t>nohy</t>
+        </is>
+      </c>
+      <c r="D172" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E172" s="3" t="inlineStr">
+        <is>
+          <t>bedna</t>
+        </is>
+      </c>
+      <c r="F172" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G172" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H172" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I172" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J172" s="3" t="inlineStr">
+        <is>
+          <t>skok</t>
+        </is>
+      </c>
+      <c r="K172" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="L172" s="4" t="inlineStr">
+        <is>
+          <t>Výskokem se dostaň na bednu a seskoč na druhou stranu. Dopadni měkce.</t>
+        </is>
+      </c>
+      <c r="M172" s="3" t="n"/>
+      <c r="N172" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="3" t="inlineStr">
+        <is>
+          <t>Veslování na kruzích</t>
+        </is>
+      </c>
+      <c r="B173" s="3" t="inlineStr">
+        <is>
+          <t>Ring row</t>
+        </is>
+      </c>
+      <c r="C173" s="3" t="inlineStr">
+        <is>
+          <t>záda</t>
+        </is>
+      </c>
+      <c r="D173" s="3" t="inlineStr">
+        <is>
+          <t>začátečník</t>
+        </is>
+      </c>
+      <c r="E173" s="3" t="inlineStr">
+        <is>
+          <t>kruhy</t>
+        </is>
+      </c>
+      <c r="F173" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G173" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H173" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I173" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J173" s="3" t="inlineStr">
+        <is>
+          <t>tah</t>
+        </is>
+      </c>
+      <c r="K173" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="L173" s="4" t="inlineStr">
+        <is>
+          <t>Drž kruhy, nakloň se dozadu a přitáhni hrudník ke kruhům. Tělo v linii.</t>
+        </is>
+      </c>
+      <c r="M173" s="3" t="n"/>
+      <c r="N173" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="3" t="inlineStr">
+        <is>
+          <t>Kliky na kruzích</t>
+        </is>
+      </c>
+      <c r="B174" s="3" t="inlineStr">
+        <is>
+          <t>Ring push-up</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>hrudník</t>
+        </is>
+      </c>
+      <c r="D174" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E174" s="3" t="inlineStr">
+        <is>
+          <t>kruhy</t>
+        </is>
+      </c>
+      <c r="F174" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G174" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H174" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I174" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J174" s="3" t="inlineStr">
+        <is>
+          <t>tlak</t>
+        </is>
+      </c>
+      <c r="K174" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L174" s="4" t="inlineStr">
+        <is>
+          <t>Ruce na kruzích, tělo v linii, spusť hrudník mezi kruhy. Vytlač zpět.</t>
+        </is>
+      </c>
+      <c r="M174" s="3" t="n"/>
+      <c r="N174" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="3" t="inlineStr">
+        <is>
+          <t>Dipy na kruzích</t>
+        </is>
+      </c>
+      <c r="B175" s="3" t="inlineStr">
+        <is>
+          <t>Ring dips</t>
+        </is>
+      </c>
+      <c r="C175" s="3" t="inlineStr">
+        <is>
+          <t>paže</t>
+        </is>
+      </c>
+      <c r="D175" s="3" t="inlineStr">
+        <is>
+          <t>expert</t>
+        </is>
+      </c>
+      <c r="E175" s="3" t="inlineStr">
+        <is>
+          <t>kruhy</t>
+        </is>
+      </c>
+      <c r="F175" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G175" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H175" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I175" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J175" s="3" t="inlineStr">
+        <is>
+          <t>tlak</t>
+        </is>
+      </c>
+      <c r="K175" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="L175" s="4" t="inlineStr">
+        <is>
+          <t>Ve vzporu na kruzích se spusť dolů s lokty u těla. Vytlač zpět.</t>
+        </is>
+      </c>
+      <c r="M175" s="3" t="n"/>
+      <c r="N175" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="3" t="inlineStr">
+        <is>
+          <t>Muscle-up na kruzích</t>
+        </is>
+      </c>
+      <c r="B176" s="3" t="inlineStr">
+        <is>
+          <t>Ring muscle-up</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="inlineStr">
+        <is>
+          <t>celé tělo</t>
+        </is>
+      </c>
+      <c r="D176" s="3" t="inlineStr">
+        <is>
+          <t>expert</t>
+        </is>
+      </c>
+      <c r="E176" s="3" t="inlineStr">
+        <is>
+          <t>kruhy</t>
+        </is>
+      </c>
+      <c r="F176" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G176" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H176" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I176" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J176" s="3" t="inlineStr">
+        <is>
+          <t>tah</t>
+        </is>
+      </c>
+      <c r="K176" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L176" s="4" t="inlineStr">
+        <is>
+          <t>Z výmyku přitáhni kruhy a převeď se do vzporu. Pak se vytlač nahoru.</t>
+        </is>
+      </c>
+      <c r="M176" s="3" t="n"/>
+      <c r="N176" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="3" t="inlineStr">
+        <is>
+          <t>Přítah s hrudníkem k hrazdě</t>
+        </is>
+      </c>
+      <c r="B177" s="3" t="inlineStr">
+        <is>
+          <t>Chest-to-bar pull-up</t>
+        </is>
+      </c>
+      <c r="C177" s="3" t="inlineStr">
+        <is>
+          <t>záda</t>
+        </is>
+      </c>
+      <c r="D177" s="3" t="inlineStr">
+        <is>
+          <t>expert</t>
+        </is>
+      </c>
+      <c r="E177" s="3" t="inlineStr">
+        <is>
+          <t>hrazda</t>
+        </is>
+      </c>
+      <c r="F177" s="3" t="inlineStr">
+        <is>
+          <t>uvnitř</t>
+        </is>
+      </c>
+      <c r="G177" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H177" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I177" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J177" s="3" t="inlineStr">
+        <is>
+          <t>tah</t>
+        </is>
+      </c>
+      <c r="K177" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="L177" s="4" t="inlineStr">
+        <is>
+          <t>Přitáhni se výbušně tak, aby se hrudník dotkl hrazdy. Dolů pod kontrolou.</t>
+        </is>
+      </c>
+      <c r="M177" s="3" t="n"/>
+      <c r="N177" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="3" t="inlineStr">
+        <is>
+          <t>Kipping přítahy</t>
+        </is>
+      </c>
+      <c r="B178" s="3" t="inlineStr">
+        <is>
+          <t>Kipping pull-up</t>
+        </is>
+      </c>
+      <c r="C178" s="3" t="inlineStr">
+        <is>
+          <t>záda</t>
+        </is>
+      </c>
+      <c r="D178" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E178" s="3" t="inlineStr">
+        <is>
+          <t>hrazda</t>
+        </is>
+      </c>
+      <c r="F178" s="3" t="inlineStr">
+        <is>
+          <t>uvnitř</t>
+        </is>
+      </c>
+      <c r="G178" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H178" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I178" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J178" s="3" t="inlineStr">
+        <is>
+          <t>tah</t>
+        </is>
+      </c>
+      <c r="K178" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="L178" s="4" t="inlineStr">
+        <is>
+          <t>Rozhoupej tělo a švihem přitáhni bradu nad hrazdu.</t>
+        </is>
+      </c>
+      <c r="M178" s="3" t="n"/>
+      <c r="N178" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="3" t="inlineStr">
+        <is>
+          <t>Kolena k loktům</t>
+        </is>
+      </c>
+      <c r="B179" s="3" t="inlineStr">
+        <is>
+          <t>Knees to elbows</t>
+        </is>
+      </c>
+      <c r="C179" s="3" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="D179" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E179" s="3" t="inlineStr">
+        <is>
+          <t>hrazda</t>
+        </is>
+      </c>
+      <c r="F179" s="3" t="inlineStr">
+        <is>
+          <t>uvnitř</t>
+        </is>
+      </c>
+      <c r="G179" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H179" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I179" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J179" s="3" t="inlineStr">
+        <is>
+          <t>jiné</t>
+        </is>
+      </c>
+      <c r="K179" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="L179" s="4" t="inlineStr">
+        <is>
+          <t>Ve visu přitáhni kolena k loktům. Pomoz si švihem z ramen.</t>
+        </is>
+      </c>
+      <c r="M179" s="3" t="n"/>
+      <c r="N179" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="3" t="inlineStr">
+        <is>
+          <t>Zvedání kolen ve visu</t>
+        </is>
+      </c>
+      <c r="B180" s="3" t="inlineStr">
+        <is>
+          <t>Hanging knee raise</t>
+        </is>
+      </c>
+      <c r="C180" s="3" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="D180" s="3" t="inlineStr">
+        <is>
+          <t>začátečník</t>
+        </is>
+      </c>
+      <c r="E180" s="3" t="inlineStr">
+        <is>
+          <t>hrazda</t>
+        </is>
+      </c>
+      <c r="F180" s="3" t="inlineStr">
+        <is>
+          <t>uvnitř</t>
+        </is>
+      </c>
+      <c r="G180" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H180" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I180" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J180" s="3" t="inlineStr">
+        <is>
+          <t>jiné</t>
+        </is>
+      </c>
+      <c r="K180" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="L180" s="4" t="inlineStr">
+        <is>
+          <t>Ve visu zvedni kolena k hrudi. Nekývej se.</t>
+        </is>
+      </c>
+      <c r="M180" s="3" t="n"/>
+      <c r="N180" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="3" t="inlineStr">
+        <is>
+          <t>Šplhání po laně</t>
+        </is>
+      </c>
+      <c r="B181" s="3" t="inlineStr">
+        <is>
+          <t>Rope climb</t>
+        </is>
+      </c>
+      <c r="C181" s="3" t="inlineStr">
+        <is>
+          <t>záda</t>
+        </is>
+      </c>
+      <c r="D181" s="3" t="inlineStr">
+        <is>
+          <t>expert</t>
+        </is>
+      </c>
+      <c r="E181" s="3" t="inlineStr">
+        <is>
+          <t>šplhací lano</t>
+        </is>
+      </c>
+      <c r="F181" s="3" t="inlineStr">
+        <is>
+          <t>uvnitř</t>
+        </is>
+      </c>
+      <c r="G181" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H181" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I181" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J181" s="3" t="inlineStr">
+        <is>
+          <t>tah</t>
+        </is>
+      </c>
+      <c r="K181" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="L181" s="4" t="inlineStr">
+        <is>
+          <t>Šplhej po laně nahoru pomocí rukou a nohou. Dolů pod kontrolou.</t>
+        </is>
+      </c>
+      <c r="M181" s="3" t="n"/>
+      <c r="N181" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="3" t="inlineStr">
+        <is>
+          <t>Kliky ve stoji na rukou</t>
+        </is>
+      </c>
+      <c r="B182" s="3" t="inlineStr">
+        <is>
+          <t>Handstand push-up</t>
+        </is>
+      </c>
+      <c r="C182" s="3" t="inlineStr">
+        <is>
+          <t>ramena</t>
+        </is>
+      </c>
+      <c r="D182" s="3" t="inlineStr">
+        <is>
+          <t>expert</t>
+        </is>
+      </c>
+      <c r="E182" s="3" t="inlineStr">
+        <is>
+          <t>vlastní váha</t>
+        </is>
+      </c>
+      <c r="F182" s="3" t="inlineStr">
+        <is>
+          <t>uvnitř</t>
+        </is>
+      </c>
+      <c r="G182" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H182" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I182" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J182" s="3" t="inlineStr">
+        <is>
+          <t>tlak</t>
+        </is>
+      </c>
+      <c r="K182" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="L182" s="4" t="inlineStr">
+        <is>
+          <t>Ve stoji na rukou u zdi ohni lokty a vytlač se zpět.</t>
+        </is>
+      </c>
+      <c r="M182" s="3" t="n"/>
+      <c r="N182" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="3" t="inlineStr">
+        <is>
+          <t>Chůze po zdi</t>
+        </is>
+      </c>
+      <c r="B183" s="3" t="inlineStr">
+        <is>
+          <t>Wall walk</t>
+        </is>
+      </c>
+      <c r="C183" s="3" t="inlineStr">
+        <is>
+          <t>celé tělo</t>
+        </is>
+      </c>
+      <c r="D183" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E183" s="3" t="inlineStr">
+        <is>
+          <t>vlastní váha</t>
+        </is>
+      </c>
+      <c r="F183" s="3" t="inlineStr">
+        <is>
+          <t>uvnitř</t>
+        </is>
+      </c>
+      <c r="G183" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H183" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I183" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J183" s="3" t="inlineStr">
+        <is>
+          <t>jiné</t>
+        </is>
+      </c>
+      <c r="K183" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="L183" s="4" t="inlineStr">
+        <is>
+          <t>Z lehu na břiše se rukama šplhej po zdi nahoru. Pak zpět.</t>
+        </is>
+      </c>
+      <c r="M183" s="3" t="n"/>
+      <c r="N183" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="3" t="inlineStr">
+        <is>
+          <t>Houpání v dutém hřbetu</t>
+        </is>
+      </c>
+      <c r="B184" s="3" t="inlineStr">
+        <is>
+          <t>Hollow rock</t>
+        </is>
+      </c>
+      <c r="C184" s="3" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="D184" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E184" s="3" t="inlineStr">
+        <is>
+          <t>vlastní váha</t>
+        </is>
+      </c>
+      <c r="F184" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G184" s="3" t="inlineStr">
+        <is>
+          <t>Tabata, CrossFit</t>
+        </is>
+      </c>
+      <c r="H184" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I184" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J184" s="3" t="inlineStr">
+        <is>
+          <t>jiné</t>
+        </is>
+      </c>
+      <c r="K184" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="L184" s="4" t="inlineStr">
+        <is>
+          <t>V pozici dutého hřbetu se kývej tam a zpět. Bedra přitlač k zemi.</t>
+        </is>
+      </c>
+      <c r="M184" s="3" t="n"/>
+      <c r="N184" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="3" t="inlineStr">
+        <is>
+          <t>Sklapovačka do V</t>
+        </is>
+      </c>
+      <c r="B185" s="3" t="inlineStr">
+        <is>
+          <t>V-up</t>
+        </is>
+      </c>
+      <c r="C185" s="3" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="D185" s="3" t="inlineStr">
+        <is>
+          <t>začátečník</t>
+        </is>
+      </c>
+      <c r="E185" s="3" t="inlineStr">
+        <is>
+          <t>vlastní váha</t>
+        </is>
+      </c>
+      <c r="F185" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G185" s="3" t="inlineStr">
+        <is>
+          <t>Tabata, CrossFit</t>
+        </is>
+      </c>
+      <c r="H185" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I185" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J185" s="3" t="inlineStr">
+        <is>
+          <t>jiné</t>
+        </is>
+      </c>
+      <c r="K185" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="L185" s="4" t="inlineStr">
+        <is>
+          <t>Vleže zvedni současně trup a nohy do tvaru V. Ruce natáhni k chodidlům.</t>
+        </is>
+      </c>
+      <c r="M185" s="3" t="n"/>
+      <c r="N185" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="3" t="inlineStr">
+        <is>
+          <t>Sed-leh na GHD</t>
+        </is>
+      </c>
+      <c r="B186" s="3" t="inlineStr">
+        <is>
+          <t>GHD sit-up</t>
+        </is>
+      </c>
+      <c r="C186" s="3" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="D186" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E186" s="3" t="inlineStr">
+        <is>
+          <t>GHD</t>
+        </is>
+      </c>
+      <c r="F186" s="3" t="inlineStr">
+        <is>
+          <t>uvnitř</t>
+        </is>
+      </c>
+      <c r="G186" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H186" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I186" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J186" s="3" t="inlineStr">
+        <is>
+          <t>jiné</t>
+        </is>
+      </c>
+      <c r="K186" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="L186" s="4" t="inlineStr">
+        <is>
+          <t>Nohy zajištěné, spusť trup dozadu a vrať se do sedu. Plynule.</t>
+        </is>
+      </c>
+      <c r="M186" s="3" t="n"/>
+      <c r="N186" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="3" t="inlineStr">
+        <is>
+          <t>Záklony na GHD</t>
+        </is>
+      </c>
+      <c r="B187" s="3" t="inlineStr">
+        <is>
+          <t>GHD hip extension</t>
+        </is>
+      </c>
+      <c r="C187" s="3" t="inlineStr">
+        <is>
+          <t>záda</t>
+        </is>
+      </c>
+      <c r="D187" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E187" s="3" t="inlineStr">
+        <is>
+          <t>GHD</t>
+        </is>
+      </c>
+      <c r="F187" s="3" t="inlineStr">
+        <is>
+          <t>uvnitř</t>
+        </is>
+      </c>
+      <c r="G187" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H187" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I187" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J187" s="3" t="inlineStr">
+        <is>
+          <t>záklon/předklon</t>
+        </is>
+      </c>
+      <c r="K187" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="L187" s="4" t="inlineStr">
+        <is>
+          <t>Na GHD se předkloň a zvedni trup do roviny. Hýždě napnuté.</t>
+        </is>
+      </c>
+      <c r="M187" s="3" t="n"/>
+      <c r="N187" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="3" t="inlineStr">
+        <is>
+          <t>Tlačení saní</t>
+        </is>
+      </c>
+      <c r="B188" s="3" t="inlineStr">
+        <is>
+          <t>Sled push</t>
+        </is>
+      </c>
+      <c r="C188" s="3" t="inlineStr">
+        <is>
+          <t>nohy</t>
+        </is>
+      </c>
+      <c r="D188" s="3" t="inlineStr">
+        <is>
+          <t>začátečník</t>
+        </is>
+      </c>
+      <c r="E188" s="3" t="inlineStr">
+        <is>
+          <t>sáně</t>
+        </is>
+      </c>
+      <c r="F188" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G188" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H188" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I188" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J188" s="3" t="inlineStr">
+        <is>
+          <t>tlak</t>
+        </is>
+      </c>
+      <c r="K188" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="L188" s="4" t="inlineStr">
+        <is>
+          <t>Tlač sáně v nízké poloze dopředu. Záda rovná, pohyb vychází z nohou.</t>
+        </is>
+      </c>
+      <c r="M188" s="3" t="n"/>
+      <c r="N188" s="3" t="inlineStr">
+        <is>
+          <t>metry</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="3" t="inlineStr">
+        <is>
+          <t>Tažení saní</t>
+        </is>
+      </c>
+      <c r="B189" s="3" t="inlineStr">
+        <is>
+          <t>Sled pull</t>
+        </is>
+      </c>
+      <c r="C189" s="3" t="inlineStr">
+        <is>
+          <t>záda</t>
+        </is>
+      </c>
+      <c r="D189" s="3" t="inlineStr">
+        <is>
+          <t>pokročilý</t>
+        </is>
+      </c>
+      <c r="E189" s="3" t="inlineStr">
+        <is>
+          <t>sáně</t>
+        </is>
+      </c>
+      <c r="F189" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G189" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H189" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I189" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J189" s="3" t="inlineStr">
+        <is>
+          <t>tah</t>
+        </is>
+      </c>
+      <c r="K189" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="L189" s="4" t="inlineStr">
+        <is>
+          <t>Zapřený couvej a táhni sáně k sobě. Chodidla pevně.</t>
+        </is>
+      </c>
+      <c r="M189" s="3" t="n"/>
+      <c r="N189" s="3" t="inlineStr">
+        <is>
+          <t>metry</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="3" t="inlineStr">
+        <is>
+          <t>Zdvih medicinbalu do dřepu</t>
+        </is>
+      </c>
+      <c r="B190" s="3" t="inlineStr">
+        <is>
+          <t>Med ball clean</t>
+        </is>
+      </c>
+      <c r="C190" s="3" t="inlineStr">
+        <is>
+          <t>celé tělo</t>
+        </is>
+      </c>
+      <c r="D190" s="3" t="inlineStr">
+        <is>
+          <t>začátečník</t>
+        </is>
+      </c>
+      <c r="E190" s="3" t="inlineStr">
+        <is>
+          <t>medicinbal</t>
+        </is>
+      </c>
+      <c r="F190" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G190" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H190" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I190" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J190" s="3" t="inlineStr">
+        <is>
+          <t>dřep</t>
+        </is>
+      </c>
+      <c r="K190" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="L190" s="4" t="inlineStr">
+        <is>
+          <t>Míč na zemi, zvedni ho do dřepu a vstaň s ním u hrudi.</t>
+        </is>
+      </c>
+      <c r="M190" s="3" t="n"/>
+      <c r="N190" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="3" t="inlineStr">
+        <is>
+          <t>Sed-leh s hodem medicinbalu</t>
+        </is>
+      </c>
+      <c r="B191" s="3" t="inlineStr">
+        <is>
+          <t>Med ball sit-up throw</t>
+        </is>
+      </c>
+      <c r="C191" s="3" t="inlineStr">
+        <is>
+          <t>core</t>
+        </is>
+      </c>
+      <c r="D191" s="3" t="inlineStr">
+        <is>
+          <t>začátečník</t>
+        </is>
+      </c>
+      <c r="E191" s="3" t="inlineStr">
+        <is>
+          <t>medicinbal</t>
+        </is>
+      </c>
+      <c r="F191" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G191" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H191" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I191" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J191" s="3" t="inlineStr">
+        <is>
+          <t>jiné</t>
+        </is>
+      </c>
+      <c r="K191" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="L191" s="4" t="inlineStr">
+        <is>
+          <t>Vleže s míčem v rukou se posaď a hoď míč do zdi. Chyť a zpět.</t>
+        </is>
+      </c>
+      <c r="M191" s="3" t="n"/>
+      <c r="N191" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="3" t="inlineStr">
+        <is>
+          <t>Zdvih kotouče nad hlavu</t>
+        </is>
+      </c>
+      <c r="B192" s="3" t="inlineStr">
+        <is>
+          <t>Plate ground to overhead</t>
+        </is>
+      </c>
+      <c r="C192" s="3" t="inlineStr">
+        <is>
+          <t>celé tělo</t>
+        </is>
+      </c>
+      <c r="D192" s="3" t="inlineStr">
+        <is>
+          <t>začátečník</t>
+        </is>
+      </c>
+      <c r="E192" s="3" t="inlineStr">
+        <is>
+          <t>kotouče</t>
+        </is>
+      </c>
+      <c r="F192" s="3" t="inlineStr">
+        <is>
+          <t>obojí</t>
+        </is>
+      </c>
+      <c r="G192" s="3" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+      <c r="H192" s="3" t="inlineStr">
+        <is>
+          <t>hlavní</t>
+        </is>
+      </c>
+      <c r="I192" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J192" s="3" t="inlineStr">
+        <is>
+          <t>dřep</t>
+        </is>
+      </c>
+      <c r="K192" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="L192" s="4" t="inlineStr">
+        <is>
+          <t>Kotouč zvedni ze země nad hlavu jedním plynulým pohybem. Záda rovná.</t>
+        </is>
+      </c>
+      <c r="M192" s="3" t="n"/>
+      <c r="N192" s="3" t="inlineStr">
+        <is>
+          <t>opakování</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N148"/>
+  <autoFilter ref="A1:N192"/>
   <dataValidations count="5">
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"nohy,záda,core,hrudník,ramena,paže,celé tělo"</formula1>
@@ -9981,12 +12797,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10005,6 +12823,16 @@
           <t>pocet_cviku</t>
         </is>
       </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>cf_nazev</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>zobrazit_v</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -10037,6 +12865,11 @@
         <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A3&amp;"*")</f>
         <v/>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Tabata, TRX</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -10053,6 +12886,16 @@
         <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A4&amp;"*")</f>
         <v/>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>kettlebell</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Tabata, TRX, CrossFit</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -10069,6 +12912,16 @@
         <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A5&amp;"*")</f>
         <v/>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>dumbbell</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Tabata, TRX, CrossFit</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -10085,6 +12938,16 @@
         <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A6&amp;"*")</f>
         <v/>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>band</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Tabata, TRX, CrossFit</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -10101,6 +12964,16 @@
         <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A7&amp;"*")</f>
         <v/>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>med ball</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Tabata, TRX, CrossFit</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -10117,6 +12990,16 @@
         <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A8&amp;"*")</f>
         <v/>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>jump rope</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Tabata, TRX, CrossFit</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -10133,6 +13016,16 @@
         <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A9&amp;"*")</f>
         <v/>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>BOX</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Tabata, TRX, CrossFit</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -10149,6 +13042,16 @@
         <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A10&amp;"*")</f>
         <v/>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>pull-up bar</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Tabata, TRX, CrossFit</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -10165,6 +13068,11 @@
         <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A11&amp;"*")</f>
         <v/>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Tabata, TRX</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -10181,6 +13089,16 @@
         <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A12&amp;"*")</f>
         <v/>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>barbell</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Tabata, TRX, CrossFit</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -10197,6 +13115,16 @@
         <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A13&amp;"*")</f>
         <v/>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>row</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Tabata, TRX, CrossFit</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -10213,6 +13141,16 @@
         <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A14&amp;"*")</f>
         <v/>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>SkiErg</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Tabata, TRX, CrossFit</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -10229,6 +13167,16 @@
         <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A15&amp;"*")-COUNTIF(Cviky!$E$2:$E$500,"*echo bike*")</f>
         <v/>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>bike</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Tabata, TRX, CrossFit</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -10245,6 +13193,16 @@
         <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A16&amp;"*")</f>
         <v/>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>echo bike</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Tabata, TRX, CrossFit</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -10261,6 +13219,16 @@
         <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A17&amp;"*")</f>
         <v/>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>sandbag</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Tabata, TRX, CrossFit</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -10277,6 +13245,11 @@
         <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A18&amp;"*")</f>
         <v/>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Tabata, TRX</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -10293,6 +13266,16 @@
         <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A19&amp;"*")</f>
         <v/>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>plates</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Tabata, TRX, CrossFit</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -10309,6 +13292,11 @@
         <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A20&amp;"*")</f>
         <v/>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Tabata, TRX</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -10325,18 +13313,148 @@
         <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A21&amp;"*")</f>
         <v/>
       </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Tabata, TRX</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
         <is>
+          <t>kruhy</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>Gymnastické kruhy.</t>
+        </is>
+      </c>
+      <c r="C22" s="6">
+        <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A22&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>rings</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>sáně</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Sáně na tlačení a tažení (sled).</t>
+        </is>
+      </c>
+      <c r="C23" s="6">
+        <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A23&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>sled</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>lavice</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Plochá lavice.</t>
+        </is>
+      </c>
+      <c r="C24" s="6">
+        <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A24&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>bench</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>GHD</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Lavice na cviky GHD.</t>
+        </is>
+      </c>
+      <c r="C25" s="6">
+        <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A25&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>GHD</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>šplhací lano</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Lano na šplhání.</t>
+        </is>
+      </c>
+      <c r="C26" s="6">
+        <f>COUNTIF(Cviky!$E$2:$E$500,"*"&amp;A26&amp;"*")</f>
+        <v/>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>rope</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>CrossFit</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>Poznámka: podložka není pomůcka (trénink s ní nepočítá). Počty zahrnují shodu textu; názvy v listu Cviky musí být přesně podle tohoto číselníku.</t>
         </is>
       </c>
-      <c r="B22" s="6" t="n"/>
-      <c r="C22" s="6" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>